<commit_message>
Deploying to gh-pages from @ Sameerakhan05/pdd-testing@08dcfcc0e31811e71bf1adb72e3511706540e0c0 🚀
</commit_message>
<xml_diff>
--- a/reports/history/build-3/Execution_Summary.xlsx
+++ b/reports/history/build-3/Execution_Summary.xlsx
@@ -22,13 +22,13 @@
     <t>Build Number</t>
   </si>
   <si>
-    <t>1</t>
+    <t>3</t>
   </si>
   <si>
     <t>Execution Date</t>
   </si>
   <si>
-    <t>2026-06-24T06:58:41.248Z</t>
+    <t>2026-06-24T07:42:24.164Z</t>
   </si>
   <si>
     <t>Total Cases</t>
@@ -475,7 +475,7 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>496</v>
+        <v>502</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -483,7 +483,7 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -491,7 +491,7 @@
         <v>9</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>